<commit_message>
🔍 Clipping update 2026-03-22: 27 Artikel (8 neu)
</commit_message>
<xml_diff>
--- a/output/20260322_MK_2026_DACH_Clipping_Report___Analysis.xlsx
+++ b/output/20260322_MK_2026_DACH_Clipping_Report___Analysis.xlsx
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -483,7 +483,7 @@
     <row r="4"/>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46103.42117907047</v>
+        <v>46103.42788746305</v>
       </c>
     </row>
     <row r="8">
@@ -525,21 +525,21 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>FONDS exklusiv</t>
+          <t>Moneycab</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Private Credit-Debatte entfacht</t>
+          <t>Nicht nur Öl: Wo der Iran-Konflikt Emerging Markets wirklich trifft</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -552,7 +552,7 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
+          <t>https://www.moneycab.com/finanz/nicht-nur-oel-wo-der-iran-konflikt-emerging-markets-wirklich-trifft/</t>
         </is>
       </c>
     </row>
@@ -562,12 +562,12 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
+          <t>FONDS exklusiv</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Anlageklasse</t>
+          <t>Private Credit-Debatte entfacht</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -577,7 +577,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>Print &amp; Online</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
@@ -585,22 +585,22 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
+          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>46085</v>
+        <v>46097</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>markteinblicke.de</t>
+          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
+          <t>Mikrofinanz als Anlageklasse</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -610,15 +610,15 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print &amp; Online</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
+          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
         </is>
       </c>
     </row>
@@ -628,12 +628,12 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>gruenderkueche.de</t>
+          <t>markteinblicke.de</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
+          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -647,26 +647,26 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
+          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>46083</v>
+        <v>46085</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>altii.de</t>
+          <t>gruenderkueche.de</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
+          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -680,26 +680,26 @@
         </is>
       </c>
       <c r="F13" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
+          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>46077</v>
+        <v>46083</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>dfpa.info</t>
+          <t>altii.de</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -713,26 +713,26 @@
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
+          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>46076</v>
+        <v>46077</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>exxecnews.org</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -750,27 +750,27 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
+          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>46069</v>
+        <v>46076</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>Börsen-Kurier</t>
+          <t>exxecnews.org</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
+          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -781,20 +781,24 @@
       <c r="F16" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="4" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>46067</v>
+        <v>46071</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>finanznachrichten.de</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Mikrofinanz: Besonderheit Anleihen mit festem Zins</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -812,27 +816,27 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
+          <t>https://www.dfpa.info/interview/mikrofinanz-besonderheit-anleihen-mit-festem-zins.html</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>46067</v>
+        <v>46069</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>bondguide.de</t>
+          <t>Börsen-Kurier</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -843,11 +847,7 @@
       <c r="F18" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
-        </is>
-      </c>
+      <c r="G18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
@@ -855,12 +855,12 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>geldmeisterin.com</t>
+          <t>finanznachrichten.de</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -878,27 +878,27 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
+          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>46057</v>
+        <v>46067</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>bondguide.de</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -911,27 +911,27 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
+          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>46055</v>
+        <v>46067</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Payoff</t>
+          <t>geldmeisterin.com</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
+          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -944,56 +944,60 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
+          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>46049</v>
+        <v>46057</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Markt Einblicke</t>
+          <t>investrends.ch</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F22" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="4" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>46044</v>
+        <v>46055</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Frankfurter Allgemeine Zeitung</t>
+          <t>Payoff</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
+          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1002,64 +1006,60 @@
         </is>
       </c>
       <c r="F23" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
+          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>46038</v>
+        <v>46049</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>E-fundresearch</t>
+          <t>Markt Einblicke</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
+          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
-        </is>
-      </c>
+      <c r="G24" s="4" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>46035</v>
+        <v>46044</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>Frankfurter Allgemeine Zeitung</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
+          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -1072,27 +1072,27 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
+          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>46029</v>
+        <v>46038</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>Markt Einblicke</t>
+          <t>E-fundresearch</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1105,27 +1105,27 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
+          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>46028</v>
+        <v>46035</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>portfolio institutionell</t>
+          <t>Finews</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Große Wirkung mit kleinen Krediten</t>
+          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -1138,7 +1138,271 @@
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
+          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>46029</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Markt Einblicke</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>46028</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>portfolio institutionell</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Große Wirkung mit kleinen Krediten</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
           <t>https://www.portfolio-institutionell.de/grosse-wirkung-mit-kleinen-krediten/</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>46000</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>investrends.ch</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>Neue Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>https://investrends.ch/aktuell/investments/neue-managementgesellschaft-fur-den-impact-fonds-alternative/</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Moneycab</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>MK Global Kapital wird per 1. Januar Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>https://www.moneycab.com/finanz/mk-global-kapital-wird-per-1-januar-managementgesellschaft-fuer-den-impact-fonds-alternative/</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>45997</v>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>bondguide.de</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>Mikro Kapital Management: Impact Investing ist kein Charity</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bondguide.de/topnews/mikro-kapital-management-impact-investing-ist-kein-charity/</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>Finews</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>Johannes Feist über Mikrofinanzen: Sollten vom hohen Ross herunterkommen</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>https://www.finews.ch/news/finanzplatz/70147-mikro-capital-johannes-feist-kuenstliche-intelligenz-blockchain-rumaenien-europa-mikrofinanzen-finanzplatz-schweiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>45973</v>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>investrends.ch</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>Mikrofinanz ist Private Debt mit direkter Verbindung zur Realwirtschaft</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>https://investrends.ch/aktuell/investments/mikrofinanz-ist-private-debt-mit-direkter-verbindung-zur-realwirtschaft/</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>45848</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Handelszeitung</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>Zwischen ESG-Müdigkeit und Wirkungsanspruch</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.handelszeitung.ch/specials/nachhaltiges-investieren-2024/zwischen-esg-mudigkeit-und-wirkungsanspruch-841576</t>
         </is>
       </c>
     </row>
@@ -1156,7 +1420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1177,7 +1441,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Source: Sheet '2026 Clippings' (A9:G27)</t>
+          <t>Source: Sheet '2026 Clippings' (A9:G35)</t>
         </is>
       </c>
     </row>
@@ -1195,7 +1459,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>19</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -1205,7 +1469,7 @@
         </is>
       </c>
       <c r="B6" s="10" t="n">
-        <v>46028</v>
+        <v>45848</v>
       </c>
     </row>
     <row r="7">
@@ -1215,7 +1479,7 @@
         </is>
       </c>
       <c r="B7" s="10" t="n">
-        <v>46097</v>
+        <v>46100</v>
       </c>
     </row>
     <row r="8">
@@ -1225,7 +1489,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -1284,18 +1548,18 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>0.2631578947368421</v>
+        <v>0.2592592592592592</v>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
-          <t>2026-01</t>
+          <t>2025-07</t>
         </is>
       </c>
       <c r="F12" s="8" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1305,144 +1569,174 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0.7368421052631579</v>
+        <v>0.7407407407407407</v>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t>2026-02</t>
+          <t>2025-11</t>
         </is>
       </c>
       <c r="F13" s="8" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="E14" s="8" t="inlineStr">
         <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="F14" s="8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="F15" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="E17" s="8" t="inlineStr">
+        <is>
           <t>2026-03</t>
         </is>
       </c>
-      <c r="F14" s="8" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="F17" s="8" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Clippings by Country</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E22" s="7" t="inlineStr">
         <is>
           <t>Clippings by Type</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="9" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Country</t>
         </is>
       </c>
-      <c r="B20" s="9" t="inlineStr">
+      <c r="B23" s="9" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C23" s="9" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E23" s="9" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
-      <c r="G20" s="9" t="inlineStr">
+      <c r="G23" s="9" t="inlineStr">
         <is>
           <t>Share</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C21" s="11" t="n">
-        <v>0.1578947368421053</v>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F21" s="8" t="n">
-        <v>17</v>
-      </c>
-      <c r="G21" s="11" t="n">
-        <v>0.8947368421052632</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="B24" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="C24" s="11" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="n">
+        <v>25</v>
+      </c>
+      <c r="G24" s="11" t="n">
+        <v>0.9259259259259259</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n">
-        <v>14</v>
-      </c>
-      <c r="C22" s="11" t="n">
-        <v>0.7368421052631579</v>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
+      <c r="B25" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="C25" s="11" t="n">
+        <v>0.5925925925925926</v>
+      </c>
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Print</t>
         </is>
       </c>
-      <c r="F22" s="8" t="n">
+      <c r="F25" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="11" t="n">
-        <v>0.05263157894736842</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="G25" s="11" t="n">
+        <v>0.03703703703703703</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>DACH</t>
         </is>
       </c>
-      <c r="B23" s="8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C23" s="11" t="n">
-        <v>0.1052631578947368</v>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
+      <c r="B26" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" s="11" t="n">
+        <v>0.07407407407407407</v>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
         <is>
           <t>Print &amp; Online</t>
         </is>
       </c>
-      <c r="F23" s="8" t="n">
+      <c r="F26" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="G23" s="11" t="n">
-        <v>0.05263157894736842</v>
+      <c r="G26" s="11" t="n">
+        <v>0.03703703703703703</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
4 neue Artikel + erweiterte Suche (Gastkommentare, cash-online, swissfinanceai, institutional-money)
</commit_message>
<xml_diff>
--- a/output/20260322_MK_2026_DACH_Clipping_Report___Analysis.xlsx
+++ b/output/20260322_MK_2026_DACH_Clipping_Report___Analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -465,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -483,7 +483,7 @@
     <row r="4"/>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46103.4944777921</v>
+        <v>46103.52625287509</v>
       </c>
     </row>
     <row r="8">
@@ -558,16 +558,16 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
-        <v>46097</v>
+        <v>46100</v>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>FONDS exklusiv</t>
+          <t>Institutional Money</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>Private Credit-Debatte entfacht</t>
+          <t>Was der Iran-Schock fuer Emerging Markets veraendert</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -581,26 +581,26 @@
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
+          <t>https://www.institutional-money.com/news/maerkte/headline/was-der-iran-schock-fuer-emerging-markets-veraendert-249420</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>46097</v>
+        <v>46098</v>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
+          <t>finanznachrichten.de</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Anlageklasse</t>
+          <t>Private Credit ist nicht gleich Private Credit: Wo die Risiken wirklich liegen</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -610,7 +610,7 @@
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>Print &amp; Online</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F11" s="4" t="n">
@@ -618,22 +618,22 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
+          <t>https://www.finanznachrichten.de/nachrichten-2026-03/67998176-private-credit-ist-nicht-gleich-private-credit-wo-die-risiken-wirklich-liegen-144.htm</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="n">
-        <v>46085</v>
+        <v>46098</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>markteinblicke.de</t>
+          <t>cash-online.de</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
+          <t>Gastkommentar: Der blinde Fleck der Private-Credit-Debatte</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -647,26 +647,26 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
+          <t>https://www.cash-online.de/a/gastkommentar-der-blinde-fleck-der-private-credit-debatte-713724/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="n">
-        <v>46085</v>
+        <v>46097</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>gruenderkueche.de</t>
+          <t>FONDS exklusiv</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
+          <t>Private Credit-Debatte entfacht</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -684,22 +684,22 @@
       </c>
       <c r="G13" s="4" t="inlineStr">
         <is>
-          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
+          <t>https://www.fondsexklusiv.de/private-credit-debatte-entfacht/</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n">
-        <v>46083</v>
+        <v>46097</v>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>altii.de</t>
+          <t>Kreditwesen (Verlagsgruppe Knapp-Richardi)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
+          <t>Mikrofinanz als Anlageklasse</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -709,35 +709,35 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print &amp; Online</t>
         </is>
       </c>
       <c r="F14" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
+          <t>https://www.kreditwesen.de/kreditwesen/themenschwerpunkte/aufsaetze/mikrofinanz-anlageklasse-id107511.html</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="n">
-        <v>46077</v>
+        <v>46091</v>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>dfpa.info</t>
+          <t>Swiss Finance AI</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Warum tokenisierte Anleihen mehr sind als ein Trend</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
@@ -750,22 +750,22 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
+          <t>https://www.swissfinanceai.ch/blog/swiss-finance/warum-tokenisierte-anleihen-mehr-sind-als-ein-trend</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="n">
-        <v>46076</v>
+        <v>46085</v>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>exxecnews.org</t>
+          <t>markteinblicke.de</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
+          <t>Tokenisierte Anleihen: Mehr Governance erforderlich</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -779,26 +779,26 @@
         </is>
       </c>
       <c r="F16" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
+          <t>https://markteinblicke.de/128943/2026/03/tokenisierte-anleihen-mehr-governance-erforderlich/</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="n">
-        <v>46071</v>
+        <v>46085</v>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>dfpa.info</t>
+          <t>gruenderkueche.de</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz: Besonderheit Anleihen mit festem Zins</t>
+          <t>Weltfrauentag: Unternehmerinnen fehlt weiterhin der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -816,27 +816,27 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>https://www.dfpa.info/interview/mikrofinanz-besonderheit-anleihen-mit-festem-zins.html</t>
+          <t>https://www.gruenderkueche.de/news/finanzen-news/weltfrauentag-unternehmerinnen-fehlt-weiterhin-der-zugang-zu-kapital/</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="n">
-        <v>46069</v>
+        <v>46083</v>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Börsen-Kurier</t>
+          <t>altii.de</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
+          <t>Unternehmerinnen fehlt weltweit der Zugang zu Kapital</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -845,22 +845,26 @@
         </is>
       </c>
       <c r="F18" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="4" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>https://www.altii.de/edai-71550571-cb6c-4c09-93da-bd99b822c245/</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="n">
-        <v>46067</v>
+        <v>46077</v>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>finanznachrichten.de</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -878,22 +882,22 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
+          <t>https://www.dfpa.info/top-story/wenn-geschaeftsbanken-passen-helfen-mikrofinanzfonds.html</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="n">
-        <v>46067</v>
+        <v>46076</v>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>bondguide.de</t>
+          <t>exxecnews.org</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
+          <t>Teil I: Wenn Geschäftsbanken passen, helfen Mikrofinanzfonds</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -911,22 +915,22 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
+          <t>https://exxecnews.org/wp-content/uploads/2026/02/Ausgabe-05_2026.pdf</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="n">
-        <v>46067</v>
+        <v>46071</v>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>geldmeisterin.com</t>
+          <t>dfpa.info</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
+          <t>Mikrofinanz: Besonderheit Anleihen mit festem Zins</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -944,27 +948,27 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
+          <t>https://www.dfpa.info/interview/mikrofinanz-besonderheit-anleihen-mit-festem-zins.html</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="n">
-        <v>46057</v>
+        <v>46069</v>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>Börsen-Kurier</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
+          <t>Privates Kapital für noch nicht entwickelte Märkte</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -975,29 +979,25 @@
       <c r="F22" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
-        </is>
-      </c>
+      <c r="G22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="n">
-        <v>46055</v>
+        <v>46067</v>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Payoff</t>
+          <t>finanznachrichten.de</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
@@ -1010,22 +1010,22 @@
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
+          <t>https://www.finanznachrichten.de/nachrichten-2026-02/67704129-security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen-144.htm</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="n">
-        <v>46049</v>
+        <v>46067</v>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Markt Einblicke</t>
+          <t>bondguide.de</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
+          <t>Security Conference München 2026: öffentliche Mittel als Hebel nutzen</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -1035,26 +1035,30 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Print</t>
+          <t>Online</t>
         </is>
       </c>
       <c r="F24" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="4" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bondguide.de/topnews/security-conference-muenchen-2026-oeffentliche-mittel-als-hebel-nutzen/</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="n">
-        <v>46044</v>
+        <v>46067</v>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Frankfurter Allgemeine Zeitung</t>
+          <t>geldmeisterin.com</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
+          <t>Mikrokredite gerade jetzt zur Risikostreuung</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1068,31 +1072,31 @@
         </is>
       </c>
       <c r="F25" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
+          <t>https://www.geldmeisterin.com/index.php/2026/02/14/mikrokredite-gerade-jetzt-zur-risikostreuung/</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="n">
-        <v>46038</v>
+        <v>46057</v>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>E-fundresearch</t>
+          <t>investrends.ch</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
+          <t>Private Debt: Warum Prozesse wichtiger sind als Prognosen</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>DACH</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -1105,22 +1109,22 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
+          <t>https://investrends.ch/aktuell/investments/private-debt-warum-prozesse-wichtiger-sind-als-prognosen/</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="n">
-        <v>46035</v>
+        <v>46055</v>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>Payoff</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
+          <t>Mikrofinanz als Private Debt: Besicherte KMU-Kredite statt «Entwicklungshilfe»</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1134,17 +1138,17 @@
         </is>
       </c>
       <c r="F27" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27" s="4" t="inlineStr">
         <is>
-          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
+          <t>https://www.payoff.ch/news/mikrofinanz-als-private-debt-besicherte-kmu-kredite-statt-entwicklungshilfe</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="n">
-        <v>46029</v>
+        <v>46049</v>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
@@ -1163,30 +1167,26 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>Online</t>
+          <t>Print</t>
         </is>
       </c>
       <c r="F28" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
-        </is>
-      </c>
+      <c r="G28" s="4" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="3" t="n">
-        <v>46028</v>
+        <v>46044</v>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>portfolio institutionell</t>
+          <t>Frankfurter Allgemeine Zeitung</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Große Wirkung mit kleinen Krediten</t>
+          <t>Beim Klimaschutz mehr Marktwirtschaft wagen</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1204,27 +1204,27 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>https://www.portfolio-institutionell.de/grosse-wirkung-mit-kleinen-krediten/</t>
+          <t>https://www.faz.net/pro/weltwirtschaft/klima-ressourcen/klimapolitik-sollte-auf-mikrofinanzierung-statt-grossprojekte-setzen-accg-200431361.html</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="n">
-        <v>46000</v>
+        <v>46038</v>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>investrends.ch</t>
+          <t>E-fundresearch</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>Neue Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+          <t>Umfrage: Welche Chancen und Risiken Experten 2026 in den Private Markets sehen</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>DACH</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
@@ -1237,22 +1237,22 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/neue-managementgesellschaft-fur-den-impact-fonds-alternative/</t>
+          <t>https://e-fundresearch.com/funds/artikel/57840-umfrage-welche-chancen-und-risiken-experten-2026-in-den-private-markets-sehen?page=5</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="n">
-        <v>45999</v>
+        <v>46035</v>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Moneycab</t>
+          <t>Finews</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>MK Global Kapital wird per 1. Januar Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+          <t>Start 2026: Disziplin als Renditequelle bei KMU-Private Debt</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1266,26 +1266,26 @@
         </is>
       </c>
       <c r="F31" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G31" s="4" t="inlineStr">
         <is>
-          <t>https://www.moneycab.com/finanz/mk-global-kapital-wird-per-1-januar-managementgesellschaft-fuer-den-impact-fonds-alternative/</t>
+          <t>https://www.finews.ch/news/finanzplatz/70792-start2026-assetmanagement-mk-global-kapital-michele-mattioda-privat-debt-kmu-mikro</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n">
-        <v>45997</v>
+        <v>46029</v>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>bondguide.de</t>
+          <t>Markt Einblicke</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>Mikro Kapital Management: Impact Investing ist kein Charity</t>
+          <t>Mikrofinanzanleihen 2026: Stabile Renditen aus der Realwirtschaft</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1303,27 +1303,27 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>https://www.bondguide.de/topnews/mikro-kapital-management-impact-investing-ist-kein-charity/</t>
+          <t>https://markteinblicke.de/127407/2026/01/mikrofinanzanleihen-2026-stabile-renditen-aus-der-realwirtschaft/</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="n">
-        <v>45985</v>
+        <v>46028</v>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Finews</t>
+          <t>portfolio institutionell</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>Johannes Feist über Mikrofinanzen: Sollten vom hohen Ross herunterkommen</t>
+          <t>Große Wirkung mit kleinen Krediten</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>CH</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
@@ -1336,13 +1336,13 @@
       </c>
       <c r="G33" s="4" t="inlineStr">
         <is>
-          <t>https://www.finews.ch/news/finanzplatz/70147-mikro-capital-johannes-feist-kuenstliche-intelligenz-blockchain-rumaenien-europa-mikrofinanzen-finanzplatz-schweiz</t>
+          <t>https://www.portfolio-institutionell.de/grosse-wirkung-mit-kleinen-krediten/</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="n">
-        <v>45973</v>
+        <v>46000</v>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>Mikrofinanz ist Private Debt mit direkter Verbindung zur Realwirtschaft</t>
+          <t>Neue Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1369,38 +1369,170 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>https://investrends.ch/aktuell/investments/mikrofinanz-ist-private-debt-mit-direkter-verbindung-zur-realwirtschaft/</t>
+          <t>https://investrends.ch/aktuell/investments/neue-managementgesellschaft-fur-den-impact-fonds-alternative/</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="n">
+        <v>45999</v>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Moneycab</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>MK Global Kapital wird per 1. Januar Managementgesellschaft für den Impact-Fonds ALTERNATIVE</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>https://www.moneycab.com/finanz/mk-global-kapital-wird-per-1-januar-managementgesellschaft-fuer-den-impact-fonds-alternative/</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>45997</v>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>bondguide.de</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>Mikro Kapital Management: Impact Investing ist kein Charity</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>https://www.bondguide.de/topnews/mikro-kapital-management-impact-investing-ist-kein-charity/</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>45985</v>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>Finews</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>Johannes Feist über Mikrofinanzen: Sollten vom hohen Ross herunterkommen</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>https://www.finews.ch/news/finanzplatz/70147-mikro-capital-johannes-feist-kuenstliche-intelligenz-blockchain-rumaenien-europa-mikrofinanzen-finanzplatz-schweiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>45973</v>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>investrends.ch</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>Mikrofinanz ist Private Debt mit direkter Verbindung zur Realwirtschaft</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>CH</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>https://investrends.ch/aktuell/investments/mikrofinanz-ist-private-debt-mit-direkter-verbindung-zur-realwirtschaft/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
         <v>45848</v>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B39" s="4" t="inlineStr">
         <is>
           <t>Handelszeitung</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>Zwischen ESG-Müdigkeit und Wirkungsanspruch</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D39" s="4" t="inlineStr">
         <is>
           <t>CH</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>Online</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="n">
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>Online</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G39" s="4" t="inlineStr">
         <is>
           <t>https://www.handelszeitung.ch/specials/nachhaltiges-investieren-2024/zwischen-esg-mudigkeit-und-wirkungsanspruch-841576</t>
         </is>
@@ -1441,7 +1573,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Source: Sheet '2026 Clippings' (A9:G35)</t>
+          <t>Source: Sheet '2026 Clippings' (A9:G39)</t>
         </is>
       </c>
     </row>
@@ -1459,7 +1591,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6">
@@ -1489,7 +1621,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -1548,10 +1680,10 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C12" s="11" t="n">
-        <v>0.2592592592592592</v>
+        <v>0.2580645161290323</v>
       </c>
       <c r="E12" s="8" t="inlineStr">
         <is>
@@ -1569,10 +1701,10 @@
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>0.7407407407407407</v>
+        <v>0.7419354838709677</v>
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
@@ -1620,7 +1752,7 @@
         </is>
       </c>
       <c r="F17" s="8" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="22">
@@ -1674,10 +1806,10 @@
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C24" s="11" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
@@ -1685,10 +1817,10 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="G24" s="11" t="n">
-        <v>0.9259259259259259</v>
+        <v>0.9354838709677419</v>
       </c>
     </row>
     <row r="25">
@@ -1698,10 +1830,10 @@
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C25" s="11" t="n">
-        <v>0.5925925925925926</v>
+        <v>0.6129032258064516</v>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
@@ -1712,7 +1844,7 @@
         <v>1</v>
       </c>
       <c r="G25" s="11" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.03225806451612903</v>
       </c>
     </row>
     <row r="26">
@@ -1725,7 +1857,7 @@
         <v>2</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>0.07407407407407407</v>
+        <v>0.06451612903225806</v>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
@@ -1736,7 +1868,7 @@
         <v>1</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.03225806451612903</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Excel mit Grafiken + Download-Button im Dashboard
</commit_message>
<xml_diff>
--- a/output/20260322_MK_2026_DACH_Clipping_Report___Analysis.xlsx
+++ b/output/20260322_MK_2026_DACH_Clipping_Report___Analysis.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 Clippings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analysis 2026" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -174,6 +174,226 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Clippings pro Monat</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Analysis 2026'!F11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analysis 2026'!$E$12:$E$17</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analysis 2026'!$F$12:$F$17</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Monat</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Anzahl</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Tier-Verteilung</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Analysis 2026'!B11</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analysis 2026'!$A$12:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analysis 2026'!$B$12:$B$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4320000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -483,7 +703,7 @@
     <row r="4"/>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46103.53156630162</v>
+        <v>46103.54655185567</v>
       </c>
     </row>
     <row r="8">
@@ -1873,5 +2093,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>